<commit_message>
fix(excel): reduce footer font size to 14pt across all sheets
Normalize Review/Approve title and date rows; fixed row height 18pt
instead of autofit that inflated D46/D47 to 16pt.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/01-original/project-report-template.xlsx
+++ b/01-original/project-report-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\timesheet-automation\01-original\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57814B00-786F-4E42-8F1E-C51B86D8F16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFF0244-B00A-4788-9614-DC98023E3775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="844" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -327,7 +327,7 @@
     <numFmt numFmtId="187" formatCode="[$-107041E]d\ mmm\ yy;@"/>
     <numFmt numFmtId="188" formatCode="[$-107041E]d\ mmmm\ yyyy;@"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="16"/>
       <color theme="1"/>
@@ -412,6 +412,19 @@
     <font>
       <b/>
       <sz val="16"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Angsana New"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
@@ -528,7 +541,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -663,6 +676,12 @@
     <xf numFmtId="49" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -671,6 +690,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -690,37 +721,25 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="188" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -766,7 +785,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>2339710</xdr:colOff>
+      <xdr:colOff>2343520</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>41325</xdr:rowOff>
     </xdr:to>
@@ -865,7 +884,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>2345425</xdr:colOff>
+      <xdr:colOff>2341615</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>41325</xdr:rowOff>
     </xdr:to>
@@ -917,7 +936,7 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>1215572</xdr:colOff>
       <xdr:row>43</xdr:row>
-      <xdr:rowOff>249281</xdr:rowOff>
+      <xdr:rowOff>245471</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -970,10 +989,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4CDAB55-AFE4-40D1-B170-94B5783AFBA3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6FF9192B-BE14-4808-B505-EE860F619952}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -996,7 +1015,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12819835" y="630463"/>
-          <a:ext cx="1688472" cy="1002898"/>
+          <a:ext cx="1694187" cy="1002898"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1020,10 +1039,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1">
+        <xdr:cNvPr id="5" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D2903A8-A4EF-4642-B52A-AA5230207998}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{24158FF6-6BEB-4ED9-8161-CC6936C75717}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1069,10 +1088,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{863AFCB0-79F4-4CBE-86DB-FB3C5D69740A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B5F09CE-979B-41E0-9D3E-3412F02FCD4A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1095,7 +1114,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12819835" y="630463"/>
-          <a:ext cx="1688472" cy="1002898"/>
+          <a:ext cx="1694187" cy="1002898"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1119,10 +1138,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1">
+        <xdr:cNvPr id="5" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2EACE53-5A21-443A-B9AA-1824A94B6376}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87529CF4-78F7-439E-8CED-82B1DCC7C59A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1168,10 +1187,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB638D5D-379C-4A03-A16A-D7695B50D86B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DB4B827-5A3D-4828-BB17-44C5C73E352E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1194,7 +1213,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12819835" y="630463"/>
-          <a:ext cx="1688472" cy="1002898"/>
+          <a:ext cx="1694187" cy="1002898"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1218,10 +1237,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1">
+        <xdr:cNvPr id="5" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CA6248C-8E72-4AEC-AEB8-0ABC691766AB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D5FBC3F-4792-4BE0-BFF2-3B8A64E3D1D9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1267,10 +1286,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D5A521B-A570-4814-BF08-974720ADAFFA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C9BADA1-4F93-4790-87F6-CA5291DC1FDB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1293,7 +1312,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12819835" y="630463"/>
-          <a:ext cx="1688472" cy="1002898"/>
+          <a:ext cx="1694187" cy="1002898"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1317,10 +1336,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1">
+        <xdr:cNvPr id="5" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DD3232F-E5AD-4AC4-AE89-B63C5209FA1E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80454B56-CEAF-4998-8604-C5003197EE9C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1366,10 +1385,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A711A828-AA12-495F-AD2F-5E3C8B238C7D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFBFA79F-8FB1-40A7-905E-22FDFFDA6FEF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1392,7 +1411,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12819835" y="630463"/>
-          <a:ext cx="1688472" cy="1002898"/>
+          <a:ext cx="1694187" cy="1002898"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1416,10 +1435,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1">
+        <xdr:cNvPr id="5" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85288027-19DD-4DA0-8A9A-38BC2B488F19}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D13E8E41-E6DD-43AF-91F9-2CFAAC82B2A0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1465,10 +1484,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4EDFCBFB-C8C7-41ED-A0E4-2281C5F37BBE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1692E80C-C449-44AE-9A46-41C2D5A857F0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1491,7 +1510,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12819835" y="630463"/>
-          <a:ext cx="1688472" cy="1002898"/>
+          <a:ext cx="1694187" cy="1002898"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1515,10 +1534,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1">
+        <xdr:cNvPr id="5" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F188A97B-4C51-44AF-AF9B-5488060A3289}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9687B3B9-67F4-456A-A62F-81CD6761BD26}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1836,28 +1855,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="51" t="str">
+      <c r="A1" s="57" t="str">
         <f>January!A1</f>
         <v>รายงานการปฏิบัติงาน</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
     </row>
     <row r="2" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="52" t="str">
+      <c r="A2" s="58" t="str">
         <f>January!A2</f>
         <v>บริษัท ไอที ดี จำกัด</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="3"/>
@@ -1869,17 +1888,17 @@
         <f>DAY(A8)&amp;" "&amp;CHOOSE(MONTH(A8),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A8)+543&amp;" ถึง "&amp;DAY(A38)&amp;" "&amp;CHOOSE(MONTH(A38),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A38)+543</f>
         <v>1 ธันวาคม 2569 ถึง 31 ธันวาคม 2569</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="69"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="71"/>
     </row>
     <row r="4" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
@@ -1894,12 +1913,12 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="53" t="str">
+      <c r="E5" s="59" t="str">
         <f>January!E5</f>
         <v>Fast Track</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A6" s="8"/>
@@ -1923,11 +1942,11 @@
       <c r="D7" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
     </row>
     <row r="8" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A8" s="16">
@@ -1936,9 +1955,9 @@
       <c r="B8" s="12"/>
       <c r="C8" s="13"/>
       <c r="D8" s="14"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="52"/>
     </row>
     <row r="9" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A9" s="16">
@@ -1948,9 +1967,9 @@
       <c r="B9" s="12"/>
       <c r="C9" s="13"/>
       <c r="D9" s="14"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="52"/>
     </row>
     <row r="10" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A10" s="16">
@@ -1960,9 +1979,9 @@
       <c r="B10" s="12"/>
       <c r="C10" s="13"/>
       <c r="D10" s="14"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="50"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="52"/>
     </row>
     <row r="11" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A11" s="16">
@@ -1972,9 +1991,9 @@
       <c r="B11" s="12"/>
       <c r="C11" s="13"/>
       <c r="D11" s="27"/>
-      <c r="E11" s="48"/>
-      <c r="F11" s="49"/>
-      <c r="G11" s="50"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="52"/>
     </row>
     <row r="12" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A12" s="33">
@@ -2026,9 +2045,9 @@
       <c r="B15" s="12"/>
       <c r="C15" s="13"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="52"/>
     </row>
     <row r="16" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A16" s="16">
@@ -2038,9 +2057,9 @@
       <c r="B16" s="12"/>
       <c r="C16" s="13"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="52"/>
     </row>
     <row r="17" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A17" s="33">
@@ -2064,9 +2083,9 @@
       <c r="B18" s="12"/>
       <c r="C18" s="13"/>
       <c r="D18" s="14"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="49"/>
-      <c r="G18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="52"/>
     </row>
     <row r="19" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A19" s="33">
@@ -2104,9 +2123,9 @@
       <c r="B21" s="12"/>
       <c r="C21" s="13"/>
       <c r="D21" s="27"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
     </row>
     <row r="22" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A22" s="16">
@@ -2116,9 +2135,9 @@
       <c r="B22" s="12"/>
       <c r="C22" s="13"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
     </row>
     <row r="23" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A23" s="16">
@@ -2128,9 +2147,9 @@
       <c r="B23" s="12"/>
       <c r="C23" s="13"/>
       <c r="D23" s="27"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="52"/>
     </row>
     <row r="24" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A24" s="16">
@@ -2140,9 +2159,9 @@
       <c r="B24" s="12"/>
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="52"/>
     </row>
     <row r="25" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A25" s="16">
@@ -2152,9 +2171,9 @@
       <c r="B25" s="12"/>
       <c r="C25" s="13"/>
       <c r="D25" s="14"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="52"/>
     </row>
     <row r="26" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A26" s="33">
@@ -2192,9 +2211,9 @@
       <c r="B28" s="12"/>
       <c r="C28" s="13"/>
       <c r="D28" s="27"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="50"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="52"/>
     </row>
     <row r="29" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A29" s="17">
@@ -2204,9 +2223,9 @@
       <c r="B29" s="12"/>
       <c r="C29" s="13"/>
       <c r="D29" s="14"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="49"/>
-      <c r="G29" s="50"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="52"/>
     </row>
     <row r="30" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A30" s="16">
@@ -2216,9 +2235,9 @@
       <c r="B30" s="12"/>
       <c r="C30" s="13"/>
       <c r="D30" s="14"/>
-      <c r="E30" s="48"/>
-      <c r="F30" s="49"/>
-      <c r="G30" s="50"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="52"/>
     </row>
     <row r="31" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A31" s="16">
@@ -2228,9 +2247,9 @@
       <c r="B31" s="12"/>
       <c r="C31" s="13"/>
       <c r="D31" s="27"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="52"/>
     </row>
     <row r="32" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A32" s="16">
@@ -2240,9 +2259,9 @@
       <c r="B32" s="12"/>
       <c r="C32" s="13"/>
       <c r="D32" s="14"/>
-      <c r="E32" s="48"/>
-      <c r="F32" s="49"/>
-      <c r="G32" s="50"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="52"/>
     </row>
     <row r="33" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A33" s="33">
@@ -2280,9 +2299,9 @@
       <c r="B35" s="12"/>
       <c r="C35" s="13"/>
       <c r="D35" s="27"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="50"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="52"/>
     </row>
     <row r="36" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A36" s="16">
@@ -2292,9 +2311,9 @@
       <c r="B36" s="12"/>
       <c r="C36" s="13"/>
       <c r="D36" s="14"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="49"/>
-      <c r="G36" s="50"/>
+      <c r="E36" s="50"/>
+      <c r="F36" s="51"/>
+      <c r="G36" s="52"/>
     </row>
     <row r="37" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A37" s="16">
@@ -2304,9 +2323,9 @@
       <c r="B37" s="12"/>
       <c r="C37" s="13"/>
       <c r="D37" s="14"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="49"/>
-      <c r="G37" s="50"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="52"/>
     </row>
     <row r="38" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A38" s="33">
@@ -2392,68 +2411,68 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="59"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="59"/>
+      <c r="E44" s="48"/>
       <c r="F44" s="36"/>
       <c r="G44" s="35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A45" s="58" t="str">
+    <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A45" s="54" t="str">
         <f>B5</f>
         <v xml:space="preserve">บุรพล อัศววิรุฬห์ฤทธิ์ </v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="D45" s="59" t="str">
+      <c r="B45" s="54"/>
+      <c r="D45" s="48" t="str">
         <f>January!$F43</f>
         <v>คุณสายฝน นามกูล</v>
       </c>
-      <c r="E45" s="59"/>
+      <c r="E45" s="48"/>
       <c r="F45" s="36"/>
       <c r="G45" s="36" t="str">
         <f>January!$H43</f>
         <v>คุณอัจฉรา ชัยภูมิ</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A46" s="60" t="str">
+    <row r="46" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="55" t="str">
         <f>January!$A$44</f>
         <v>Programmer</v>
       </c>
-      <c r="B46" s="60"/>
+      <c r="B46" s="55"/>
       <c r="C46" s="26"/>
-      <c r="D46" s="61" t="s">
+      <c r="D46" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="61"/>
+      <c r="E46" s="68"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.6">
+    <row r="47" spans="1:7" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A47" s="23"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
-      <c r="D47" s="62" t="s">
+      <c r="D47" s="69" t="s">
         <v>83</v>
       </c>
-      <c r="E47" s="62"/>
+      <c r="E47" s="69"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
     </row>
     <row r="48" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A48" s="23"/>
-      <c r="B48" s="57"/>
-      <c r="C48" s="57"/>
+      <c r="B48" s="53"/>
+      <c r="C48" s="53"/>
       <c r="D48" s="24"/>
       <c r="E48" s="24"/>
       <c r="F48" s="25"/>
@@ -2524,22 +2543,13 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="E35:G35"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="E37:G37"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="E7:G7"/>
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="E30:G30"/>
     <mergeCell ref="E31:G31"/>
@@ -2550,13 +2560,22 @@
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="E28:G28"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B38" xr:uid="{266C3BD5-A414-437D-8A74-48A5E9321021}">
@@ -2638,26 +2657,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
     </row>
     <row r="2" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="3"/>
@@ -2674,12 +2693,12 @@
       <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
@@ -2693,11 +2712,11 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="53" t="s">
+      <c r="E5" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A6" s="8"/>
@@ -2721,11 +2740,11 @@
       <c r="D7" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
     </row>
     <row r="8" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A8" s="33">
@@ -3101,8 +3120,8 @@
       <c r="C37" s="13"/>
       <c r="D37" s="14"/>
       <c r="E37" s="15"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="50"/>
+      <c r="F37" s="50"/>
+      <c r="G37" s="52"/>
     </row>
     <row r="38" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A38" s="33">
@@ -3119,10 +3138,10 @@
       <c r="G38" s="46"/>
     </row>
     <row r="39" spans="1:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A39" s="54" t="s">
+      <c r="A39" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="B39" s="56"/>
+      <c r="B39" s="62"/>
       <c r="C39" s="18">
         <f>SUM(C8:C38)</f>
         <v>0</v>
@@ -3205,61 +3224,61 @@
       </c>
     </row>
     <row r="44" spans="1:8" s="26" customFormat="1" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="48" t="s">
         <v>86</v>
       </c>
-      <c r="B44" s="59"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="59"/>
+      <c r="E44" s="48"/>
       <c r="F44" s="36"/>
       <c r="G44" s="35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A45" s="58" t="str">
+    <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A45" s="54" t="str">
         <f>B5</f>
         <v xml:space="preserve">บุรพล อัศววิรุฬห์ฤทธิ์ </v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="D45" s="59" t="str">
+      <c r="B45" s="54"/>
+      <c r="D45" s="48" t="str">
         <f>January!$F43</f>
         <v>คุณสายฝน นามกูล</v>
       </c>
-      <c r="E45" s="59"/>
+      <c r="E45" s="48"/>
       <c r="F45" s="36"/>
       <c r="G45" s="36" t="str">
         <f>January!$H43</f>
         <v>คุณอัจฉรา ชัยภูมิ</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A46" s="60" t="str">
+    <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="55" t="str">
         <f>January!$A$44</f>
         <v>Programmer</v>
       </c>
-      <c r="B46" s="60"/>
+      <c r="B46" s="55"/>
       <c r="C46" s="26"/>
-      <c r="D46" s="61" t="s">
+      <c r="D46" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="61"/>
+      <c r="E46" s="56"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="47" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A47" s="23"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
-      <c r="D47" s="62" t="s">
+      <c r="D47" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="E47" s="62"/>
+      <c r="E47" s="49"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
     </row>
@@ -3310,27 +3329,6 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E7:G7"/>
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="F16:G16"/>
@@ -3344,6 +3342,27 @@
     <mergeCell ref="F27:G27"/>
     <mergeCell ref="F28:G28"/>
     <mergeCell ref="F26:G26"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8 B10:B11 B17:B18 B24:B25 B31:B32 B38" xr:uid="{8E689AAC-4CCD-406A-B21F-86181782FF32}">
@@ -3379,28 +3398,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="65" t="str">
+      <c r="A1" s="66" t="str">
         <f>January!A1</f>
         <v>รายงานการปฏิบัติงาน</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
     </row>
     <row r="2" spans="1:9" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="52" t="str">
+      <c r="A2" s="58" t="str">
         <f>January!A2</f>
         <v>บริษัท ไอที ดี จำกัด</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:9" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="3"/>
@@ -3412,17 +3431,17 @@
         <f>DAY(A8)&amp;" "&amp;CHOOSE(MONTH(A8),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A8)+543&amp;" ถึง "&amp;DAY(A37)&amp;" "&amp;CHOOSE(MONTH(A37),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A37)+543</f>
         <v>1 มิถุนายน 2569 ถึง 30 มิถุนายน 2569</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="69"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="71"/>
     </row>
     <row r="4" spans="1:9" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
@@ -3437,12 +3456,12 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="53" t="str">
+      <c r="E5" s="59" t="str">
         <f>January!E5</f>
         <v>Fast Track</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A6" s="8"/>
@@ -3466,11 +3485,11 @@
       <c r="D7" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
     </row>
     <row r="8" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A8" s="33">
@@ -3500,11 +3519,11 @@
       <c r="D9" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="66" t="s">
+      <c r="E9" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="49"/>
-      <c r="G9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="52"/>
     </row>
     <row r="10" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A10" s="33">
@@ -3534,11 +3553,11 @@
       <c r="D11" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="66" t="s">
+      <c r="E11" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="49"/>
-      <c r="G11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="52"/>
     </row>
     <row r="12" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A12" s="16">
@@ -3554,11 +3573,11 @@
       <c r="D12" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="66" t="s">
+      <c r="E12" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="49"/>
-      <c r="G12" s="50"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="52"/>
     </row>
     <row r="13" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A13" s="33">
@@ -3602,11 +3621,11 @@
       <c r="D15" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="66" t="s">
+      <c r="E15" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="F15" s="49"/>
-      <c r="G15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="52"/>
     </row>
     <row r="16" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A16" s="16">
@@ -3622,11 +3641,11 @@
       <c r="D16" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="66" t="s">
+      <c r="E16" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="49"/>
-      <c r="G16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="52"/>
     </row>
     <row r="17" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A17" s="16">
@@ -3642,11 +3661,11 @@
       <c r="D17" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="66" t="s">
+      <c r="E17" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="49"/>
-      <c r="G17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="52"/>
     </row>
     <row r="18" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A18" s="16">
@@ -3662,11 +3681,11 @@
       <c r="D18" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="66" t="s">
+      <c r="E18" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="F18" s="49"/>
-      <c r="G18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="52"/>
     </row>
     <row r="19" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A19" s="16">
@@ -3682,11 +3701,11 @@
       <c r="D19" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="66" t="s">
+      <c r="E19" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="F19" s="49"/>
-      <c r="G19" s="50"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="52"/>
     </row>
     <row r="20" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A20" s="33">
@@ -3730,11 +3749,11 @@
       <c r="D22" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="66" t="s">
+      <c r="E22" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="F22" s="49"/>
-      <c r="G22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
     </row>
     <row r="23" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A23" s="16">
@@ -3750,11 +3769,11 @@
       <c r="D23" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="E23" s="66" t="s">
+      <c r="E23" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="F23" s="49"/>
-      <c r="G23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="52"/>
     </row>
     <row r="24" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A24" s="16">
@@ -3770,11 +3789,11 @@
       <c r="D24" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="E24" s="66" t="s">
+      <c r="E24" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="F24" s="49"/>
-      <c r="G24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="52"/>
     </row>
     <row r="25" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A25" s="16">
@@ -3790,11 +3809,11 @@
       <c r="D25" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="E25" s="66" t="s">
+      <c r="E25" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="F25" s="49"/>
-      <c r="G25" s="50"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="52"/>
     </row>
     <row r="26" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A26" s="16">
@@ -3810,11 +3829,11 @@
       <c r="D26" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="66" t="s">
+      <c r="E26" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="49"/>
-      <c r="G26" s="50"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="52"/>
     </row>
     <row r="27" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A27" s="33">
@@ -3858,11 +3877,11 @@
       <c r="D29" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="E29" s="66" t="s">
+      <c r="E29" s="65" t="s">
         <v>59</v>
       </c>
-      <c r="F29" s="49"/>
-      <c r="G29" s="50"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="52"/>
     </row>
     <row r="30" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A30" s="16">
@@ -3878,11 +3897,11 @@
       <c r="D30" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="E30" s="66" t="s">
+      <c r="E30" s="65" t="s">
         <v>61</v>
       </c>
-      <c r="F30" s="49"/>
-      <c r="G30" s="50"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="52"/>
     </row>
     <row r="31" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A31" s="16">
@@ -3898,11 +3917,11 @@
       <c r="D31" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="E31" s="66" t="s">
+      <c r="E31" s="65" t="s">
         <v>63</v>
       </c>
-      <c r="F31" s="49"/>
-      <c r="G31" s="50"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="52"/>
     </row>
     <row r="32" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A32" s="16">
@@ -3918,11 +3937,11 @@
       <c r="D32" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="E32" s="66" t="s">
+      <c r="E32" s="65" t="s">
         <v>65</v>
       </c>
-      <c r="F32" s="49"/>
-      <c r="G32" s="50"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="52"/>
     </row>
     <row r="33" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A33" s="16">
@@ -3938,11 +3957,11 @@
       <c r="D33" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="E33" s="66" t="s">
+      <c r="E33" s="65" t="s">
         <v>67</v>
       </c>
-      <c r="F33" s="49"/>
-      <c r="G33" s="50"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="52"/>
     </row>
     <row r="34" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A34" s="33">
@@ -3986,11 +4005,11 @@
       <c r="D36" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="E36" s="66" t="s">
+      <c r="E36" s="65" t="s">
         <v>69</v>
       </c>
-      <c r="F36" s="49"/>
-      <c r="G36" s="50"/>
+      <c r="F36" s="51"/>
+      <c r="G36" s="52"/>
     </row>
     <row r="37" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A37" s="17">
@@ -4006,11 +4025,11 @@
       <c r="D37" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="E37" s="66" t="s">
+      <c r="E37" s="65" t="s">
         <v>71</v>
       </c>
-      <c r="F37" s="49"/>
-      <c r="G37" s="50"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="52"/>
     </row>
     <row r="38" spans="1:7" ht="11.55" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A38" s="19"/>
@@ -4091,60 +4110,60 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="59"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="59"/>
+      <c r="E44" s="48"/>
       <c r="F44" s="36"/>
       <c r="G44" s="35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A45" s="58" t="str">
+    <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A45" s="54" t="str">
         <f>B5</f>
         <v xml:space="preserve">บุรพล อัศววิรุฬห์ฤทธิ์ </v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="D45" s="59" t="str">
+      <c r="B45" s="54"/>
+      <c r="D45" s="48" t="str">
         <f>January!$F43</f>
         <v>คุณสายฝน นามกูล</v>
       </c>
-      <c r="E45" s="59"/>
+      <c r="E45" s="48"/>
       <c r="F45" s="36"/>
       <c r="G45" s="36" t="str">
         <f>January!$H43</f>
         <v>คุณอัจฉรา ชัยภูมิ</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="A46" s="60" t="str">
+    <row r="46" spans="1:7" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="55" t="str">
         <f>January!$A$44</f>
         <v>Programmer</v>
       </c>
-      <c r="B46" s="60"/>
-      <c r="D46" s="61" t="s">
+      <c r="B46" s="55"/>
+      <c r="D46" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="61"/>
+      <c r="E46" s="68"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.6">
+    <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A47" s="23"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
-      <c r="D47" s="62" t="s">
+      <c r="D47" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="E47" s="62"/>
+      <c r="E47" s="69"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
     </row>
@@ -4213,22 +4232,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="E33:G33"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="D44:E44"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:F4"/>
@@ -4245,6 +4248,22 @@
     <mergeCell ref="E22:G22"/>
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="E24:G24"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="E33:G33"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="E31:G31"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B37" xr:uid="{010ABD38-6107-482D-8158-FF133F270DB6}">
@@ -4277,28 +4296,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="65" t="str">
+      <c r="A1" s="66" t="str">
         <f>January!A1</f>
         <v>รายงานการปฏิบัติงาน</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
     </row>
     <row r="2" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="52" t="str">
+      <c r="A2" s="58" t="str">
         <f>January!A2</f>
         <v>บริษัท ไอที ดี จำกัด</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="3"/>
@@ -4310,17 +4329,17 @@
         <f>DAY(A8)&amp;" "&amp;CHOOSE(MONTH(A8),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A8)+543&amp;" ถึง "&amp;DAY(A38)&amp;" "&amp;CHOOSE(MONTH(A38),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A38)+543</f>
         <v>1 กรกฎาคม 2569 ถึง 31 กรกฎาคม 2569</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="69"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="71"/>
     </row>
     <row r="4" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
@@ -4335,12 +4354,12 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="53" t="str">
+      <c r="E5" s="59" t="str">
         <f>January!E5</f>
         <v>Fast Track</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A6" s="8"/>
@@ -4364,11 +4383,11 @@
       <c r="D7" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
     </row>
     <row r="8" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A8" s="28">
@@ -4377,9 +4396,9 @@
       <c r="B8" s="12"/>
       <c r="C8" s="13"/>
       <c r="D8" s="14"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="52"/>
     </row>
     <row r="9" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A9" s="16">
@@ -4389,9 +4408,9 @@
       <c r="B9" s="12"/>
       <c r="C9" s="13"/>
       <c r="D9" s="14"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="52"/>
     </row>
     <row r="10" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A10" s="16">
@@ -4401,9 +4420,9 @@
       <c r="B10" s="12"/>
       <c r="C10" s="13"/>
       <c r="D10" s="14"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="50"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="52"/>
     </row>
     <row r="11" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A11" s="33">
@@ -4441,9 +4460,9 @@
       <c r="B13" s="12"/>
       <c r="C13" s="13"/>
       <c r="D13" s="14"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="52"/>
     </row>
     <row r="14" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A14" s="16">
@@ -4453,9 +4472,9 @@
       <c r="B14" s="12"/>
       <c r="C14" s="13"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="50"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="52"/>
     </row>
     <row r="15" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A15" s="16">
@@ -4465,9 +4484,9 @@
       <c r="B15" s="12"/>
       <c r="C15" s="13"/>
       <c r="D15" s="27"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="52"/>
     </row>
     <row r="16" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A16" s="16">
@@ -4477,9 +4496,9 @@
       <c r="B16" s="12"/>
       <c r="C16" s="13"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="52"/>
     </row>
     <row r="17" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A17" s="16">
@@ -4489,9 +4508,9 @@
       <c r="B17" s="12"/>
       <c r="C17" s="13"/>
       <c r="D17" s="14"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="52"/>
     </row>
     <row r="18" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A18" s="33">
@@ -4529,9 +4548,9 @@
       <c r="B20" s="12"/>
       <c r="C20" s="13"/>
       <c r="D20" s="27"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="52"/>
     </row>
     <row r="21" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A21" s="16">
@@ -4541,9 +4560,9 @@
       <c r="B21" s="12"/>
       <c r="C21" s="13"/>
       <c r="D21" s="14"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
     </row>
     <row r="22" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A22" s="16">
@@ -4553,9 +4572,9 @@
       <c r="B22" s="12"/>
       <c r="C22" s="13"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
     </row>
     <row r="23" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A23" s="16">
@@ -4565,9 +4584,9 @@
       <c r="B23" s="12"/>
       <c r="C23" s="13"/>
       <c r="D23" s="27"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="52"/>
     </row>
     <row r="24" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A24" s="16">
@@ -4577,9 +4596,9 @@
       <c r="B24" s="12"/>
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="52"/>
     </row>
     <row r="25" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A25" s="33">
@@ -4617,9 +4636,9 @@
       <c r="B27" s="12"/>
       <c r="C27" s="13"/>
       <c r="D27" s="14"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="52"/>
     </row>
     <row r="28" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A28" s="16">
@@ -4629,9 +4648,9 @@
       <c r="B28" s="12"/>
       <c r="C28" s="13"/>
       <c r="D28" s="14"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="50"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="52"/>
     </row>
     <row r="29" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A29" s="16">
@@ -4641,9 +4660,9 @@
       <c r="B29" s="12"/>
       <c r="C29" s="13"/>
       <c r="D29" s="14"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="49"/>
-      <c r="G29" s="50"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="52"/>
     </row>
     <row r="30" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A30" s="16">
@@ -4653,9 +4672,9 @@
       <c r="B30" s="12"/>
       <c r="C30" s="13"/>
       <c r="D30" s="14"/>
-      <c r="E30" s="48"/>
-      <c r="F30" s="49"/>
-      <c r="G30" s="50"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="52"/>
     </row>
     <row r="31" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A31" s="16">
@@ -4665,9 +4684,9 @@
       <c r="B31" s="12"/>
       <c r="C31" s="13"/>
       <c r="D31" s="27"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="52"/>
     </row>
     <row r="32" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A32" s="33">
@@ -4705,9 +4724,9 @@
       <c r="B34" s="12"/>
       <c r="C34" s="13"/>
       <c r="D34" s="14"/>
-      <c r="E34" s="48"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="52"/>
     </row>
     <row r="35" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A35" s="33">
@@ -4745,9 +4764,9 @@
       <c r="B37" s="12"/>
       <c r="C37" s="13"/>
       <c r="D37" s="14"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="49"/>
-      <c r="G37" s="50"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="52"/>
     </row>
     <row r="38" spans="1:7" ht="11.55" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A38" s="17">
@@ -4757,9 +4776,9 @@
       <c r="B38" s="12"/>
       <c r="C38" s="13"/>
       <c r="D38" s="14"/>
-      <c r="E38" s="48"/>
-      <c r="F38" s="49"/>
-      <c r="G38" s="50"/>
+      <c r="E38" s="50"/>
+      <c r="F38" s="51"/>
+      <c r="G38" s="52"/>
     </row>
     <row r="39" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A39" s="19"/>
@@ -4831,60 +4850,60 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="59"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="59"/>
+      <c r="E44" s="48"/>
       <c r="F44" s="36"/>
       <c r="G44" s="35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A45" s="58" t="str">
+    <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A45" s="54" t="str">
         <f>B5</f>
         <v xml:space="preserve">บุรพล อัศววิรุฬห์ฤทธิ์ </v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="D45" s="59" t="str">
+      <c r="B45" s="54"/>
+      <c r="D45" s="48" t="str">
         <f>January!$F43</f>
         <v>คุณสายฝน นามกูล</v>
       </c>
-      <c r="E45" s="59"/>
+      <c r="E45" s="48"/>
       <c r="F45" s="36"/>
       <c r="G45" s="36" t="str">
         <f>January!$H43</f>
         <v>คุณอัจฉรา ชัยภูมิ</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="A46" s="60" t="str">
+    <row r="46" spans="1:7" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="55" t="str">
         <f>January!$A$44</f>
         <v>Programmer</v>
       </c>
-      <c r="B46" s="60"/>
-      <c r="D46" s="61" t="s">
+      <c r="B46" s="55"/>
+      <c r="D46" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="61"/>
+      <c r="E46" s="68"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.6">
+    <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A47" s="23"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
-      <c r="D47" s="62" t="s">
+      <c r="D47" s="69" t="s">
         <v>78</v>
       </c>
-      <c r="E47" s="62"/>
+      <c r="E47" s="69"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
     </row>
@@ -4953,6 +4972,26 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E7:G7"/>
     <mergeCell ref="E9:G9"/>
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="E13:G13"/>
@@ -4966,26 +5005,6 @@
     <mergeCell ref="E21:G21"/>
     <mergeCell ref="E22:G22"/>
     <mergeCell ref="E23:G23"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="E37:G37"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B38" xr:uid="{11217B32-120A-47D5-84B7-4A5092F3DC71}">
@@ -5030,16 +5049,16 @@
       <c r="G1" s="67"/>
     </row>
     <row r="2" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="52" t="str">
+      <c r="A2" s="58" t="str">
         <f>January!A2</f>
         <v>บริษัท ไอที ดี จำกัด</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="3"/>
@@ -5051,17 +5070,17 @@
         <f>DAY(A8)&amp;" "&amp;CHOOSE(MONTH(A8),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A8)+543&amp;" ถึง "&amp;DAY(A38)&amp;" "&amp;CHOOSE(MONTH(A38),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A38)+543</f>
         <v>1 สิงหาคม 2569 ถึง 31 สิงหาคม 2569</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="69"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="71"/>
     </row>
     <row r="4" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
@@ -5076,12 +5095,12 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="53" t="str">
+      <c r="E5" s="59" t="str">
         <f>January!E5</f>
         <v>Fast Track</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A6" s="8"/>
@@ -5105,11 +5124,11 @@
       <c r="D7" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
     </row>
     <row r="8" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A8" s="33">
@@ -5146,9 +5165,9 @@
       <c r="B10" s="12"/>
       <c r="C10" s="13"/>
       <c r="D10" s="27"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="50"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="52"/>
     </row>
     <row r="11" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A11" s="16">
@@ -5158,9 +5177,9 @@
       <c r="B11" s="12"/>
       <c r="C11" s="13"/>
       <c r="D11" s="14"/>
-      <c r="E11" s="48"/>
-      <c r="F11" s="49"/>
-      <c r="G11" s="50"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="52"/>
     </row>
     <row r="12" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A12" s="16">
@@ -5170,9 +5189,9 @@
       <c r="B12" s="12"/>
       <c r="C12" s="13"/>
       <c r="D12" s="14"/>
-      <c r="E12" s="48"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="50"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="52"/>
     </row>
     <row r="13" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A13" s="16">
@@ -5182,9 +5201,9 @@
       <c r="B13" s="12"/>
       <c r="C13" s="13"/>
       <c r="D13" s="14"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="52"/>
     </row>
     <row r="14" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A14" s="16">
@@ -5194,9 +5213,9 @@
       <c r="B14" s="12"/>
       <c r="C14" s="13"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="50"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="52"/>
     </row>
     <row r="15" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A15" s="33">
@@ -5234,9 +5253,9 @@
       <c r="B17" s="12"/>
       <c r="C17" s="13"/>
       <c r="D17" s="27"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="52"/>
     </row>
     <row r="18" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A18" s="16">
@@ -5246,9 +5265,9 @@
       <c r="B18" s="12"/>
       <c r="C18" s="13"/>
       <c r="D18" s="14"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="49"/>
-      <c r="G18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="52"/>
     </row>
     <row r="19" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A19" s="33">
@@ -5272,9 +5291,9 @@
       <c r="B20" s="12"/>
       <c r="C20" s="13"/>
       <c r="D20" s="14"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="52"/>
     </row>
     <row r="21" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A21" s="16">
@@ -5284,9 +5303,9 @@
       <c r="B21" s="12"/>
       <c r="C21" s="13"/>
       <c r="D21" s="14"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
     </row>
     <row r="22" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A22" s="33">
@@ -5324,9 +5343,9 @@
       <c r="B24" s="12"/>
       <c r="C24" s="13"/>
       <c r="D24" s="27"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="52"/>
     </row>
     <row r="25" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A25" s="16">
@@ -5336,9 +5355,9 @@
       <c r="B25" s="12"/>
       <c r="C25" s="13"/>
       <c r="D25" s="14"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="52"/>
     </row>
     <row r="26" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A26" s="16">
@@ -5348,9 +5367,9 @@
       <c r="B26" s="12"/>
       <c r="C26" s="13"/>
       <c r="D26" s="14"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="52"/>
     </row>
     <row r="27" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A27" s="16">
@@ -5360,9 +5379,9 @@
       <c r="B27" s="12"/>
       <c r="C27" s="13"/>
       <c r="D27" s="27"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="52"/>
     </row>
     <row r="28" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A28" s="16">
@@ -5372,9 +5391,9 @@
       <c r="B28" s="12"/>
       <c r="C28" s="13"/>
       <c r="D28" s="14"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="50"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="52"/>
     </row>
     <row r="29" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A29" s="33">
@@ -5412,9 +5431,9 @@
       <c r="B31" s="12"/>
       <c r="C31" s="13"/>
       <c r="D31" s="27"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="52"/>
     </row>
     <row r="32" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A32" s="16">
@@ -5424,9 +5443,9 @@
       <c r="B32" s="12"/>
       <c r="C32" s="13"/>
       <c r="D32" s="14"/>
-      <c r="E32" s="48"/>
-      <c r="F32" s="49"/>
-      <c r="G32" s="50"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="52"/>
     </row>
     <row r="33" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A33" s="16">
@@ -5436,9 +5455,9 @@
       <c r="B33" s="12"/>
       <c r="C33" s="13"/>
       <c r="D33" s="14"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="50"/>
+      <c r="E33" s="50"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="52"/>
     </row>
     <row r="34" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A34" s="16">
@@ -5448,9 +5467,9 @@
       <c r="B34" s="12"/>
       <c r="C34" s="13"/>
       <c r="D34" s="14"/>
-      <c r="E34" s="48"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="52"/>
     </row>
     <row r="35" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A35" s="16">
@@ -5460,9 +5479,9 @@
       <c r="B35" s="12"/>
       <c r="C35" s="13"/>
       <c r="D35" s="27"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="50"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="52"/>
     </row>
     <row r="36" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A36" s="33">
@@ -5500,9 +5519,9 @@
       <c r="B38" s="12"/>
       <c r="C38" s="13"/>
       <c r="D38" s="13"/>
-      <c r="E38" s="48"/>
-      <c r="F38" s="49"/>
-      <c r="G38" s="50"/>
+      <c r="E38" s="50"/>
+      <c r="F38" s="51"/>
+      <c r="G38" s="52"/>
     </row>
     <row r="39" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A39" s="19"/>
@@ -5574,60 +5593,60 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="59"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="59"/>
+      <c r="E44" s="48"/>
       <c r="F44" s="36"/>
       <c r="G44" s="35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A45" s="58" t="str">
+    <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A45" s="54" t="str">
         <f>B5</f>
         <v xml:space="preserve">บุรพล อัศววิรุฬห์ฤทธิ์ </v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="D45" s="59" t="str">
+      <c r="B45" s="54"/>
+      <c r="D45" s="48" t="str">
         <f>January!$F43</f>
         <v>คุณสายฝน นามกูล</v>
       </c>
-      <c r="E45" s="59"/>
+      <c r="E45" s="48"/>
       <c r="F45" s="36"/>
       <c r="G45" s="36" t="str">
         <f>January!$H43</f>
         <v>คุณอัจฉรา ชัยภูมิ</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="A46" s="60" t="str">
+    <row r="46" spans="1:7" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="55" t="str">
         <f>January!$A$44</f>
         <v>Programmer</v>
       </c>
-      <c r="B46" s="60"/>
-      <c r="D46" s="61" t="s">
+      <c r="B46" s="55"/>
+      <c r="D46" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="61"/>
+      <c r="E46" s="68"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.6">
+    <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A47" s="23"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
-      <c r="D47" s="62" t="s">
+      <c r="D47" s="69" t="s">
         <v>79</v>
       </c>
-      <c r="E47" s="62"/>
+      <c r="E47" s="69"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
     </row>
@@ -5696,6 +5715,23 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="E14:G14"/>
     <mergeCell ref="E38:G38"/>
     <mergeCell ref="E33:G33"/>
     <mergeCell ref="E34:G34"/>
@@ -5711,23 +5747,6 @@
     <mergeCell ref="E26:G26"/>
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="E28:G28"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B38" xr:uid="{83C74234-C585-4522-A2AD-E38E4F1DA4CF}">
@@ -5760,28 +5779,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="65" t="str">
+      <c r="A1" s="66" t="str">
         <f>January!A1</f>
         <v>รายงานการปฏิบัติงาน</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
     </row>
     <row r="2" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="52" t="str">
+      <c r="A2" s="58" t="str">
         <f>January!A2</f>
         <v>บริษัท ไอที ดี จำกัด</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="3"/>
@@ -5793,17 +5812,17 @@
         <f>DAY(A8)&amp;" "&amp;CHOOSE(MONTH(A8),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A8)+543&amp;" ถึง "&amp;DAY(A37)&amp;" "&amp;CHOOSE(MONTH(A37),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A37)+543</f>
         <v>1 กันยายน 2569 ถึง 30 กันยายน 2569</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="69"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="71"/>
     </row>
     <row r="4" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
@@ -5818,12 +5837,12 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="53" t="str">
+      <c r="E5" s="59" t="str">
         <f>January!E5</f>
         <v>Fast Track</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A6" s="8"/>
@@ -5847,11 +5866,11 @@
       <c r="D7" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
     </row>
     <row r="8" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A8" s="16">
@@ -5860,9 +5879,9 @@
       <c r="B8" s="12"/>
       <c r="C8" s="13"/>
       <c r="D8" s="14"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="52"/>
     </row>
     <row r="9" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A9" s="16">
@@ -5872,9 +5891,9 @@
       <c r="B9" s="12"/>
       <c r="C9" s="13"/>
       <c r="D9" s="14"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="52"/>
     </row>
     <row r="10" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A10" s="16">
@@ -5884,9 +5903,9 @@
       <c r="B10" s="12"/>
       <c r="C10" s="13"/>
       <c r="D10" s="14"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="50"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="52"/>
     </row>
     <row r="11" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A11" s="16">
@@ -5896,9 +5915,9 @@
       <c r="B11" s="12"/>
       <c r="C11" s="13"/>
       <c r="D11" s="27"/>
-      <c r="E11" s="48"/>
-      <c r="F11" s="49"/>
-      <c r="G11" s="50"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="52"/>
     </row>
     <row r="12" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A12" s="33">
@@ -5936,9 +5955,9 @@
       <c r="B14" s="12"/>
       <c r="C14" s="13"/>
       <c r="D14" s="27"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="50"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="52"/>
     </row>
     <row r="15" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A15" s="16">
@@ -5948,9 +5967,9 @@
       <c r="B15" s="12"/>
       <c r="C15" s="13"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="52"/>
     </row>
     <row r="16" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A16" s="16">
@@ -5960,9 +5979,9 @@
       <c r="B16" s="12"/>
       <c r="C16" s="13"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="52"/>
     </row>
     <row r="17" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A17" s="16">
@@ -5972,9 +5991,9 @@
       <c r="B17" s="12"/>
       <c r="C17" s="13"/>
       <c r="D17" s="14"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="52"/>
     </row>
     <row r="18" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A18" s="16">
@@ -5984,9 +6003,9 @@
       <c r="B18" s="12"/>
       <c r="C18" s="13"/>
       <c r="D18" s="14"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="49"/>
-      <c r="G18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="52"/>
     </row>
     <row r="19" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A19" s="33">
@@ -6024,9 +6043,9 @@
       <c r="B21" s="12"/>
       <c r="C21" s="13"/>
       <c r="D21" s="27"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
     </row>
     <row r="22" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A22" s="16">
@@ -6036,9 +6055,9 @@
       <c r="B22" s="12"/>
       <c r="C22" s="13"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
     </row>
     <row r="23" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A23" s="16">
@@ -6048,9 +6067,9 @@
       <c r="B23" s="12"/>
       <c r="C23" s="13"/>
       <c r="D23" s="27"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="52"/>
     </row>
     <row r="24" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A24" s="16">
@@ -6060,9 +6079,9 @@
       <c r="B24" s="12"/>
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="52"/>
     </row>
     <row r="25" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A25" s="16">
@@ -6072,9 +6091,9 @@
       <c r="B25" s="12"/>
       <c r="C25" s="13"/>
       <c r="D25" s="14"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="52"/>
     </row>
     <row r="26" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A26" s="33">
@@ -6112,9 +6131,9 @@
       <c r="B28" s="12"/>
       <c r="C28" s="13"/>
       <c r="D28" s="27"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="50"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="52"/>
     </row>
     <row r="29" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A29" s="16">
@@ -6124,9 +6143,9 @@
       <c r="B29" s="12"/>
       <c r="C29" s="13"/>
       <c r="D29" s="14"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="49"/>
-      <c r="G29" s="50"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="52"/>
     </row>
     <row r="30" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A30" s="16">
@@ -6136,9 +6155,9 @@
       <c r="B30" s="12"/>
       <c r="C30" s="13"/>
       <c r="D30" s="14"/>
-      <c r="E30" s="48"/>
-      <c r="F30" s="49"/>
-      <c r="G30" s="50"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="52"/>
     </row>
     <row r="31" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A31" s="16">
@@ -6148,9 +6167,9 @@
       <c r="B31" s="12"/>
       <c r="C31" s="13"/>
       <c r="D31" s="27"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="52"/>
     </row>
     <row r="32" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A32" s="16">
@@ -6160,9 +6179,9 @@
       <c r="B32" s="12"/>
       <c r="C32" s="13"/>
       <c r="D32" s="14"/>
-      <c r="E32" s="48"/>
-      <c r="F32" s="49"/>
-      <c r="G32" s="50"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="52"/>
     </row>
     <row r="33" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A33" s="33">
@@ -6200,9 +6219,9 @@
       <c r="B35" s="12"/>
       <c r="C35" s="13"/>
       <c r="D35" s="27"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="50"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="52"/>
     </row>
     <row r="36" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A36" s="16">
@@ -6212,9 +6231,9 @@
       <c r="B36" s="12"/>
       <c r="C36" s="13"/>
       <c r="D36" s="14"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="49"/>
-      <c r="G36" s="50"/>
+      <c r="E36" s="50"/>
+      <c r="F36" s="51"/>
+      <c r="G36" s="52"/>
     </row>
     <row r="37" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A37" s="17">
@@ -6224,9 +6243,9 @@
       <c r="B37" s="12"/>
       <c r="C37" s="13"/>
       <c r="D37" s="14"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="49"/>
-      <c r="G37" s="50"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="52"/>
     </row>
     <row r="38" spans="1:7" ht="11.55" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A38" s="19"/>
@@ -6307,62 +6326,62 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="59"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="59"/>
+      <c r="E44" s="48"/>
       <c r="F44" s="36"/>
       <c r="G44" s="35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="A45" s="58" t="str">
+    <row r="45" spans="1:7" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A45" s="54" t="str">
         <f>B5</f>
         <v xml:space="preserve">บุรพล อัศววิรุฬห์ฤทธิ์ </v>
       </c>
-      <c r="B45" s="58"/>
+      <c r="B45" s="54"/>
       <c r="C45"/>
-      <c r="D45" s="59" t="str">
+      <c r="D45" s="48" t="str">
         <f>January!$F43</f>
         <v>คุณสายฝน นามกูล</v>
       </c>
-      <c r="E45" s="59"/>
+      <c r="E45" s="48"/>
       <c r="F45" s="36"/>
       <c r="G45" s="36" t="str">
         <f>January!$H43</f>
         <v>คุณอัจฉรา ชัยภูมิ</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A46" s="60" t="str">
+    <row r="46" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="55" t="str">
         <f>January!$A$44</f>
         <v>Programmer</v>
       </c>
-      <c r="B46" s="60"/>
+      <c r="B46" s="55"/>
       <c r="C46" s="26"/>
-      <c r="D46" s="61" t="s">
+      <c r="D46" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="61"/>
+      <c r="E46" s="68"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.6">
+    <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A47" s="23"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
-      <c r="D47" s="62" t="s">
+      <c r="D47" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="E47" s="62"/>
+      <c r="E47" s="69"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
     </row>
@@ -6422,6 +6441,24 @@
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="E8:G8"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="E35:G35"/>
     <mergeCell ref="E36:G36"/>
@@ -6438,24 +6475,6 @@
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="E18:G18"/>
     <mergeCell ref="E23:G23"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B37" xr:uid="{80CB82DC-9453-4D83-8AD0-5FFEA696200A}">
@@ -6488,28 +6507,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="51" t="str">
+      <c r="A1" s="57" t="str">
         <f>January!A1</f>
         <v>รายงานการปฏิบัติงาน</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
     </row>
     <row r="2" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="52" t="str">
+      <c r="A2" s="58" t="str">
         <f>January!A2</f>
         <v>บริษัท ไอที ดี จำกัด</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="3"/>
@@ -6521,17 +6540,17 @@
         <f>DAY(A8)&amp;" "&amp;CHOOSE(MONTH(A8),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A8)+543&amp;" ถึง "&amp;DAY(A38)&amp;" "&amp;CHOOSE(MONTH(A38),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A38)+543</f>
         <v>1 ตุลาคม 2569 ถึง 31 ตุลาคม 2569</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="69"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="71"/>
     </row>
     <row r="4" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
@@ -6546,12 +6565,12 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="53" t="str">
+      <c r="E5" s="59" t="str">
         <f>January!E5</f>
         <v>Fast Track</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A6" s="8"/>
@@ -6575,11 +6594,11 @@
       <c r="D7" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
     </row>
     <row r="8" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A8" s="28">
@@ -6588,9 +6607,9 @@
       <c r="B8" s="12"/>
       <c r="C8" s="13"/>
       <c r="D8" s="14"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="52"/>
     </row>
     <row r="9" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A9" s="16">
@@ -6600,9 +6619,9 @@
       <c r="B9" s="12"/>
       <c r="C9" s="13"/>
       <c r="D9" s="14"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="52"/>
     </row>
     <row r="10" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A10" s="33">
@@ -6640,9 +6659,9 @@
       <c r="B12" s="12"/>
       <c r="C12" s="13"/>
       <c r="D12" s="14"/>
-      <c r="E12" s="48"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="50"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="52"/>
     </row>
     <row r="13" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A13" s="16">
@@ -6652,9 +6671,9 @@
       <c r="B13" s="12"/>
       <c r="C13" s="13"/>
       <c r="D13" s="14"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="52"/>
     </row>
     <row r="14" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A14" s="16">
@@ -6664,9 +6683,9 @@
       <c r="B14" s="12"/>
       <c r="C14" s="13"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="50"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="52"/>
     </row>
     <row r="15" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A15" s="16">
@@ -6676,9 +6695,9 @@
       <c r="B15" s="12"/>
       <c r="C15" s="13"/>
       <c r="D15" s="27"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="52"/>
     </row>
     <row r="16" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A16" s="16">
@@ -6688,9 +6707,9 @@
       <c r="B16" s="12"/>
       <c r="C16" s="13"/>
       <c r="D16" s="14"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="52"/>
     </row>
     <row r="17" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A17" s="33">
@@ -6728,9 +6747,9 @@
       <c r="B19" s="12"/>
       <c r="C19" s="13"/>
       <c r="D19" s="27"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="52"/>
     </row>
     <row r="20" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A20" s="33">
@@ -6754,9 +6773,9 @@
       <c r="B21" s="12"/>
       <c r="C21" s="13"/>
       <c r="D21" s="14"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
     </row>
     <row r="22" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A22" s="16">
@@ -6766,9 +6785,9 @@
       <c r="B22" s="12"/>
       <c r="C22" s="13"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
     </row>
     <row r="23" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A23" s="16">
@@ -6778,9 +6797,9 @@
       <c r="B23" s="12"/>
       <c r="C23" s="13"/>
       <c r="D23" s="27"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="52"/>
     </row>
     <row r="24" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A24" s="33">
@@ -6818,9 +6837,9 @@
       <c r="B26" s="12"/>
       <c r="C26" s="13"/>
       <c r="D26" s="27"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="52"/>
     </row>
     <row r="27" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A27" s="16">
@@ -6830,9 +6849,9 @@
       <c r="B27" s="12"/>
       <c r="C27" s="13"/>
       <c r="D27" s="14"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="52"/>
     </row>
     <row r="28" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A28" s="16">
@@ -6842,9 +6861,9 @@
       <c r="B28" s="12"/>
       <c r="C28" s="13"/>
       <c r="D28" s="14"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="50"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="52"/>
     </row>
     <row r="29" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A29" s="16">
@@ -6854,9 +6873,9 @@
       <c r="B29" s="12"/>
       <c r="C29" s="13"/>
       <c r="D29" s="14"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="49"/>
-      <c r="G29" s="50"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="52"/>
     </row>
     <row r="30" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A30" s="33">
@@ -6908,9 +6927,9 @@
       <c r="B33" s="12"/>
       <c r="C33" s="13"/>
       <c r="D33" s="27"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="50"/>
+      <c r="E33" s="50"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="52"/>
     </row>
     <row r="34" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A34" s="16">
@@ -6920,9 +6939,9 @@
       <c r="B34" s="12"/>
       <c r="C34" s="13"/>
       <c r="D34" s="14"/>
-      <c r="E34" s="48"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="52"/>
     </row>
     <row r="35" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A35" s="16">
@@ -6932,9 +6951,9 @@
       <c r="B35" s="12"/>
       <c r="C35" s="13"/>
       <c r="D35" s="27"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="50"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="52"/>
     </row>
     <row r="36" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A36" s="16">
@@ -6944,9 +6963,9 @@
       <c r="B36" s="12"/>
       <c r="C36" s="13"/>
       <c r="D36" s="14"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="49"/>
-      <c r="G36" s="50"/>
+      <c r="E36" s="50"/>
+      <c r="F36" s="51"/>
+      <c r="G36" s="52"/>
     </row>
     <row r="37" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A37" s="16">
@@ -6956,9 +6975,9 @@
       <c r="B37" s="12"/>
       <c r="C37" s="13"/>
       <c r="D37" s="14"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="49"/>
-      <c r="G37" s="50"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="52"/>
     </row>
     <row r="38" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A38" s="33">
@@ -7044,68 +7063,68 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="59"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="59"/>
+      <c r="E44" s="48"/>
       <c r="F44" s="36"/>
       <c r="G44" s="35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A45" s="58" t="str">
+    <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A45" s="54" t="str">
         <f>B5</f>
         <v xml:space="preserve">บุรพล อัศววิรุฬห์ฤทธิ์ </v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="D45" s="59" t="str">
+      <c r="B45" s="54"/>
+      <c r="D45" s="48" t="str">
         <f>January!$F43</f>
         <v>คุณสายฝน นามกูล</v>
       </c>
-      <c r="E45" s="59"/>
+      <c r="E45" s="48"/>
       <c r="F45" s="36"/>
       <c r="G45" s="36" t="str">
         <f>January!$H43</f>
         <v>คุณอัจฉรา ชัยภูมิ</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A46" s="60" t="str">
+    <row r="46" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="55" t="str">
         <f>January!$A$44</f>
         <v>Programmer</v>
       </c>
-      <c r="B46" s="60"/>
+      <c r="B46" s="55"/>
       <c r="C46" s="26"/>
-      <c r="D46" s="61" t="s">
+      <c r="D46" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="61"/>
+      <c r="E46" s="68"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.6">
+    <row r="47" spans="1:7" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A47" s="23"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
-      <c r="D47" s="62" t="s">
+      <c r="D47" s="69" t="s">
         <v>81</v>
       </c>
-      <c r="E47" s="62"/>
+      <c r="E47" s="69"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
     </row>
     <row r="48" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A48" s="23"/>
-      <c r="B48" s="57"/>
-      <c r="C48" s="57"/>
+      <c r="B48" s="53"/>
+      <c r="C48" s="53"/>
       <c r="D48" s="24"/>
       <c r="E48" s="24"/>
       <c r="F48" s="25"/>
@@ -7176,6 +7195,23 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E16:G16"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="D47:E47"/>
@@ -7192,23 +7228,6 @@
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="E28:G28"/>
     <mergeCell ref="D44:E44"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E7:G7"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B38" xr:uid="{0370F45E-DD39-4033-823E-C93AA0E4384F}">
@@ -7241,28 +7260,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="51" t="str">
+      <c r="A1" s="57" t="str">
         <f>January!A1</f>
         <v>รายงานการปฏิบัติงาน</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
     </row>
     <row r="2" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="52" t="str">
+      <c r="A2" s="58" t="str">
         <f>January!A2</f>
         <v>บริษัท ไอที ดี จำกัด</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="3"/>
@@ -7274,17 +7293,17 @@
         <f>DAY(A8)&amp;" "&amp;CHOOSE(MONTH(A8),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A8)+543&amp;" ถึง "&amp;DAY(A37)&amp;" "&amp;CHOOSE(MONTH(A37),"มกราคม","กุมภาพันธ์","มีนาคม","เมษายน","พฤษภาคม","มิถุนายน","กรกฎาคม","สิงหาคม","กันยายน","ตุลาคม","พฤศจิกายน","ธันวาคม")&amp;" "&amp;YEAR(A37)+543</f>
         <v>1 พฤศจิกายน 2569 ถึง 30 พฤศจิกายน 2569</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="69"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="71"/>
     </row>
     <row r="4" spans="1:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.6">
@@ -7299,12 +7318,12 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="53" t="str">
+      <c r="E5" s="59" t="str">
         <f>January!E5</f>
         <v>Fast Track</v>
       </c>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A6" s="8"/>
@@ -7328,11 +7347,11 @@
       <c r="D7" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="56"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
     </row>
     <row r="8" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A8" s="33">
@@ -7355,9 +7374,9 @@
       <c r="B9" s="12"/>
       <c r="C9" s="13"/>
       <c r="D9" s="27"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="52"/>
     </row>
     <row r="10" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A10" s="16">
@@ -7367,9 +7386,9 @@
       <c r="B10" s="12"/>
       <c r="C10" s="13"/>
       <c r="D10" s="14"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="50"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="52"/>
     </row>
     <row r="11" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A11" s="16">
@@ -7379,9 +7398,9 @@
       <c r="B11" s="12"/>
       <c r="C11" s="13"/>
       <c r="D11" s="27"/>
-      <c r="E11" s="48"/>
-      <c r="F11" s="49"/>
-      <c r="G11" s="50"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="52"/>
     </row>
     <row r="12" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A12" s="16">
@@ -7391,9 +7410,9 @@
       <c r="B12" s="12"/>
       <c r="C12" s="13"/>
       <c r="D12" s="14"/>
-      <c r="E12" s="48"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="50"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="52"/>
     </row>
     <row r="13" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A13" s="16">
@@ -7403,9 +7422,9 @@
       <c r="B13" s="12"/>
       <c r="C13" s="13"/>
       <c r="D13" s="14"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="52"/>
     </row>
     <row r="14" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A14" s="33">
@@ -7443,9 +7462,9 @@
       <c r="B16" s="12"/>
       <c r="C16" s="13"/>
       <c r="D16" s="27"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="52"/>
     </row>
     <row r="17" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A17" s="16">
@@ -7455,9 +7474,9 @@
       <c r="B17" s="12"/>
       <c r="C17" s="13"/>
       <c r="D17" s="14"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="52"/>
     </row>
     <row r="18" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A18" s="16">
@@ -7467,9 +7486,9 @@
       <c r="B18" s="12"/>
       <c r="C18" s="13"/>
       <c r="D18" s="14"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="49"/>
-      <c r="G18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="52"/>
     </row>
     <row r="19" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A19" s="16">
@@ -7479,9 +7498,9 @@
       <c r="B19" s="12"/>
       <c r="C19" s="13"/>
       <c r="D19" s="27"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="52"/>
     </row>
     <row r="20" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A20" s="16">
@@ -7491,9 +7510,9 @@
       <c r="B20" s="12"/>
       <c r="C20" s="13"/>
       <c r="D20" s="14"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="52"/>
     </row>
     <row r="21" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A21" s="33">
@@ -7531,9 +7550,9 @@
       <c r="B23" s="12"/>
       <c r="C23" s="13"/>
       <c r="D23" s="27"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="52"/>
     </row>
     <row r="24" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A24" s="16">
@@ -7543,9 +7562,9 @@
       <c r="B24" s="12"/>
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="52"/>
     </row>
     <row r="25" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A25" s="16">
@@ -7555,9 +7574,9 @@
       <c r="B25" s="12"/>
       <c r="C25" s="13"/>
       <c r="D25" s="14"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="52"/>
     </row>
     <row r="26" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A26" s="16">
@@ -7567,9 +7586,9 @@
       <c r="B26" s="12"/>
       <c r="C26" s="13"/>
       <c r="D26" s="14"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="52"/>
     </row>
     <row r="27" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A27" s="16">
@@ -7579,9 +7598,9 @@
       <c r="B27" s="12"/>
       <c r="C27" s="13"/>
       <c r="D27" s="27"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="52"/>
     </row>
     <row r="28" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A28" s="33">
@@ -7619,9 +7638,9 @@
       <c r="B30" s="12"/>
       <c r="C30" s="13"/>
       <c r="D30" s="27"/>
-      <c r="E30" s="48"/>
-      <c r="F30" s="49"/>
-      <c r="G30" s="50"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="52"/>
     </row>
     <row r="31" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A31" s="16">
@@ -7631,9 +7650,9 @@
       <c r="B31" s="12"/>
       <c r="C31" s="13"/>
       <c r="D31" s="14"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="52"/>
     </row>
     <row r="32" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A32" s="16">
@@ -7643,9 +7662,9 @@
       <c r="B32" s="12"/>
       <c r="C32" s="13"/>
       <c r="D32" s="14"/>
-      <c r="E32" s="48"/>
-      <c r="F32" s="49"/>
-      <c r="G32" s="50"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="52"/>
     </row>
     <row r="33" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A33" s="16">
@@ -7655,9 +7674,9 @@
       <c r="B33" s="12"/>
       <c r="C33" s="13"/>
       <c r="D33" s="14"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="50"/>
+      <c r="E33" s="50"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="52"/>
     </row>
     <row r="34" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A34" s="16">
@@ -7667,9 +7686,9 @@
       <c r="B34" s="12"/>
       <c r="C34" s="13"/>
       <c r="D34" s="14"/>
-      <c r="E34" s="48"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="52"/>
     </row>
     <row r="35" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A35" s="33">
@@ -7707,9 +7726,9 @@
       <c r="B37" s="12"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="49"/>
-      <c r="G37" s="50"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="52"/>
     </row>
     <row r="38" spans="1:7" ht="11.55" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A38" s="19"/>
@@ -7790,60 +7809,60 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="59"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="59"/>
+      <c r="E44" s="48"/>
       <c r="F44" s="36"/>
       <c r="G44" s="35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A45" s="58" t="str">
+    <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A45" s="54" t="str">
         <f>B5</f>
         <v xml:space="preserve">บุรพล อัศววิรุฬห์ฤทธิ์ </v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="D45" s="59" t="str">
+      <c r="B45" s="54"/>
+      <c r="D45" s="48" t="str">
         <f>January!$F43</f>
         <v>คุณสายฝน นามกูล</v>
       </c>
-      <c r="E45" s="59"/>
+      <c r="E45" s="48"/>
       <c r="F45" s="36"/>
       <c r="G45" s="36" t="str">
         <f>January!$H43</f>
         <v>คุณอัจฉรา ชัยภูมิ</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="A46" s="60" t="str">
+    <row r="46" spans="1:7" s="26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A46" s="55" t="str">
         <f>January!$A$44</f>
         <v>Programmer</v>
       </c>
-      <c r="B46" s="60"/>
-      <c r="D46" s="61" t="s">
+      <c r="B46" s="55"/>
+      <c r="D46" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="61"/>
+      <c r="E46" s="68"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.6">
+    <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A47" s="23"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25"/>
-      <c r="D47" s="62" t="s">
+      <c r="D47" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="E47" s="62"/>
+      <c r="E47" s="69"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
     </row>
@@ -7912,6 +7931,23 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="E17:G17"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="E37:G37"/>
     <mergeCell ref="A46:B46"/>
@@ -7928,23 +7964,6 @@
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="E20:G20"/>
     <mergeCell ref="E16:G16"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="E27:G27"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B37" xr:uid="{CE502D94-C7D0-4625-AA55-EEC4165A3D17}">

</xml_diff>